<commit_message>
Addtion of ROS reporting templates
</commit_message>
<xml_diff>
--- a/form_reporting_templates/Form-1RC.xlsx
+++ b/form_reporting_templates/Form-1RC.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71F8A4CA-0912-420E-9927-076251F80989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="5O4euoXp3wZfikUhVbwGMfw3acpHwF0QGHqLGhqkSE4QfnoccY7VPEsDDzzEBP5NB49UT+XbcZf1lZQTbDpLFA==" workbookSaltValue="DtEOIJKZ9UKP8oWrD+QpRw==" workbookSpinCount="100000" lockStructure="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB143897-F89E-4AC8-9534-56ECFDC7AA7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="lAFjslrjGwMTJE1NUXLE5pTcATr50ZXgQDF5h+/zjiA7wioNfNjVw9nYkQ1dgkPJEq6LlnMfcg0xE0pvmT7qvw==" workbookSaltValue="GMhYgpJXEvtJ1Uf1ocN3vw==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -1440,6 +1440,7 @@
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="MPAJMHKMDh7E71vkBfNk/kd8ZSdpOJSzU53tPHgyGpVTowbGxJWEzAge5U21K78NzbmIcA20rOCSW3K6Jiov+g==" saltValue="THz5x9zEcHi/JbRcb6UtPQ==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <dataConsolidate/>
   <mergeCells count="4">
     <mergeCell ref="C25:G25"/>
     <mergeCell ref="C8:D8"/>
@@ -2607,7 +2608,7 @@
       <c r="J55" s="53"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="o/aMX/ctE+vE+3wwnBsLSp3jQR82RU8JgABtS9/SA1WckTSR/wNyQychBaXnf4BG3tOGHt0cp2lt5BgZXsneZg==" saltValue="O5OKEDbE8C45hfR0YqTPtA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="rXFGwVus8+iBeooLP73bc/W99AccTd0zyJrbKibyeAGPXI+iXfFCmh2F+C49CJwMm/IP/ta1u0hPhP7AF8b2fQ==" saltValue="AXfkDwSa/Y/9gX97HLl8Jg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="5">
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="I4:J4"/>

</xml_diff>